<commit_message>
Set Tokyo Electron to non-technical track
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C4stvb6MmoWgtSQhmF5884
</commit_message>
<xml_diff>
--- a/internship/インターン・本選考_企業比較.xlsx
+++ b/internship/インターン・本選考_企業比較.xlsx
@@ -2241,24 +2241,24 @@
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>技術営業</t>
+          <t>半導体・電機メーカー</t>
         </is>
       </c>
       <c r="D21" s="20" t="inlineStr">
         <is>
-          <t>（候補）東京エレクトロン</t>
+          <t>東京エレクトロン</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>技術営業／FE</t>
+          <t>文系職（営業・管理系）</t>
         </is>
       </c>
       <c r="F21" s="21" t="n">
         <v>1300</v>
       </c>
       <c r="G21" s="19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="O21" s="20" t="inlineStr">
         <is>
-          <t>技術営業で給料高い枠の候補</t>
+          <t>文系職で応募。年収は全社平均の目安</t>
         </is>
       </c>
     </row>
@@ -7749,7 +7749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B10"/>
+  <dimension ref="B1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="2" max="2"/>
@@ -7814,12 +7814,19 @@
     <row r="9">
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>商社</t>
+          <t>半導体・電機メーカー</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>商社</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>その他</t>
         </is>

</xml_diff>

<commit_message>
Update Tokyo Electron salary estimate for non-technical track
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C4stvb6MmoWgtSQhmF5884
</commit_message>
<xml_diff>
--- a/internship/インターン・本選考_企業比較.xlsx
+++ b/internship/インターン・本選考_企業比較.xlsx
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>1300</v>
+        <v>950</v>
       </c>
       <c r="G21" s="19" t="n">
         <v>4</v>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="O21" s="20" t="inlineStr">
         <is>
-          <t>文系職で応募。年収は全社平均の目安</t>
+          <t>文系職で応募。950=口コミの営業職平均935万・総合職965万（OpenWork）。有報の全社平均は1,354万（2025/3期・平均43.5歳）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add survey sheet on administrative-track hiring ratio at chemical/materials makers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C4stvb6MmoWgtSQhmF5884
</commit_message>
<xml_diff>
--- a/internship/インターン・本選考_企業比較.xlsx
+++ b/internship/インターン・本選考_企業比較.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="サマリー" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="企業一覧" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="リスト" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="事務系比率調査" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="リスト" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'企業一覧'!$A$4:$O$200</definedName>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="m/d"/>
     <numFmt numFmtId="165" formatCode="0&quot;日&quot;;&quot;期限切れ&quot;;&quot;今日&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,8 +69,14 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +101,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -123,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -190,6 +202,28 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -7749,6 +7783,600 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:I26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>化学・素材メーカーの事務系（文系職）採用比率 調査</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Web検索で見つかった公開データ（就活サイト・各社採用ページ）を集計。2026年9月時点。人数は青字＝入力値なので、正確な数字が分かれば上書きすると再計算されます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>会社</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>年度</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>事務系
+(名)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>技術系
+(名)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>事務系
+比率</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>データの種類</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>注意点</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>住友化学</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="E6" s="28" t="n">
+        <v>36</v>
+      </c>
+      <c r="F6" s="9">
+        <f>D6+E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="29">
+        <f>IF(F6=0,"",D6/F6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>実績</t>
+        </is>
+      </c>
+      <c r="I6" s="27" t="inlineStr">
+        <is>
+          <t>総合職（クリエイティブスタッフ）のみ。事務系21名の内訳は学士20・修士1。2021年度は全体で文系32・理系81</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>信越化学工業</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>2020-2026計</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>83</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>529</v>
+      </c>
+      <c r="F7" s="18">
+        <f>D7+E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="30">
+        <f>IF(F7=0,"",D7/F7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>実績</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>7年分の合計（一般職は除く）。2025年は事務15・技術89</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>三井化学</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>97</v>
+      </c>
+      <c r="F8" s="18">
+        <f>D8+E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="30">
+        <f>IF(F8=0,"",D8/F8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>実績</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>東レ</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>61</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>118</v>
+      </c>
+      <c r="F9" s="18">
+        <f>D9+E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="30">
+        <f>IF(F9=0,"",D9/F9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>実績</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>118/61を男女別とする情報もあり要確認。2024年は事務62・技術141</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>日産化学</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>2023-2025計</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>95</v>
+      </c>
+      <c r="F10" s="18">
+        <f>D10+E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="30">
+        <f>IF(F10=0,"",D10/F10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>実績</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>3年分の合計</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>AGC</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>26</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>128</v>
+      </c>
+      <c r="F11" s="18">
+        <f>D11+E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="30">
+        <f>IF(F11=0,"",D11/F11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>実績</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>2026年予定は事務22・技術90</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>日東電工</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>105</v>
+      </c>
+      <c r="F12" s="18">
+        <f>D12+E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="30">
+        <f>IF(F12=0,"",D12/F12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>実績</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>事務系＝営業管理系</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>住友ベークライト</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>2022-2024計</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>31</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>57</v>
+      </c>
+      <c r="F13" s="18">
+        <f>D13+E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="30">
+        <f>IF(F13=0,"",D13/F13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>実績</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>3年分の合計</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>JFEスチール</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>2023-2025計</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>143</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>341</v>
+      </c>
+      <c r="F14" s="18">
+        <f>D14+E14</f>
+        <v/>
+      </c>
+      <c r="G14" s="30">
+        <f>IF(F14=0,"",D14/F14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>実績</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>3年分の合計</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>東ソー</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>例年</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="E15" s="19" t="n">
+        <v>80</v>
+      </c>
+      <c r="F15" s="18">
+        <f>D15+E15</f>
+        <v/>
+      </c>
+      <c r="G15" s="30">
+        <f>IF(F15=0,"",D15/F15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="18" t="inlineStr">
+        <is>
+          <t>概数</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>「例年 事務20・技術80前後」という記載</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>レゾナック</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>例年</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>120</v>
+      </c>
+      <c r="F16" s="18">
+        <f>D16+E16</f>
+        <v/>
+      </c>
+      <c r="G16" s="30">
+        <f>IF(F16=0,"",D16/F16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>概数</t>
+        </is>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>「全体約150・文系職約30」という記載</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>クラレ</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>2026募集</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="F17" s="18">
+        <f>D17+E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="30">
+        <f>IF(F17=0,"",D17/F17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
+          <t>募集人数</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>募集 事務15〜25・技術40〜50 の中央値</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>全社合計（人数で加重）</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="32">
+        <f>SUM(D6:D17)</f>
+        <v/>
+      </c>
+      <c r="E19" s="32">
+        <f>SUM(E6:E17)</f>
+        <v/>
+      </c>
+      <c r="F19" s="32">
+        <f>D19+E19</f>
+        <v/>
+      </c>
+      <c r="G19" s="33">
+        <f>D19/F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="31" t="inlineStr">
+        <is>
+          <t>会社ごと比率の中央値</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="32" t="n"/>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="33">
+        <f>MEDIAN(G6:G17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="31" t="inlineStr">
+        <is>
+          <t>会社ごと比率の最小〜最大</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="32" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="33">
+        <f>TEXT(MIN(G6:G17),"0%")&amp;"〜"&amp;TEXT(MAX(G6:G17),"0%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>・「事務系の中の文系・理系の割合」を公開している会社は見つからなかったため、事務系（≒文系職）が採用全体に占める割合で比較しています。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>・事務系には理系の学生も応募できるので、実際に文系の学生が入れる枠は事務系の人数より少し少なくなります。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>・住友化学の事務系21名は学士20名・修士1名で、ほとんどが学部卒でした（文系の学生が多い可能性が高いと推測）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>・出典：各社採用サイト、マイナビ・リクナビ、ワンキャリア、unistyle などの検索結果（一部は就活サイトによる二次情報）。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7756,77 +8384,77 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="34" t="inlineStr">
         <is>
           <t>業界（プルダウンの選択肢。追加・変更OK）</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="27" t="inlineStr">
+      <c r="B2" s="35" t="inlineStr">
         <is>
           <t>コンサル</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="27" t="inlineStr">
+      <c r="B3" s="35" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="35" t="inlineStr">
         <is>
           <t>人材・広告</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="35" t="inlineStr">
         <is>
           <t>鉄鋼・素材</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>化学</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="35" t="inlineStr">
         <is>
           <t>プラント・エンジ</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>技術営業</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="35" t="inlineStr">
         <is>
           <t>半導体・電機メーカー</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>商社</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>その他</t>
         </is>

</xml_diff>

<commit_message>
Add table of published liberal-arts/science ratios for administrative-track hires
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C4stvb6MmoWgtSQhmF5884
</commit_message>
<xml_diff>
--- a/internship/インターン・本選考_企業比較.xlsx
+++ b/internship/インターン・本選考_企業比較.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="m/d"/>
     <numFmt numFmtId="165" formatCode="0&quot;日&quot;;&quot;期限切れ&quot;;&quot;今日&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +74,12 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="7">
@@ -135,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -226,6 +232,7 @@
     <xf numFmtId="9" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -7783,7 +7790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I26"/>
+  <dimension ref="B2:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8363,6 +8370,207 @@
       <c r="B26" s="2" t="inlineStr">
         <is>
           <t>・出典：各社採用サイト、マイナビ・リクナビ、ワンキャリア、unistyle などの検索結果（一部は就活サイトによる二次情報）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="34" t="inlineStr">
+        <is>
+          <t>② 事務系の文系・理系の内訳が分かる会社（公開数値）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>会社</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>年度</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>文系</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>理系</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>理系
+比率</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>区分</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>注意点</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>富士フイルムビジネスイノベーション</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>最新</t>
+        </is>
+      </c>
+      <c r="D31" s="28" t="n">
+        <v>85</v>
+      </c>
+      <c r="E31" s="28" t="n">
+        <v>15</v>
+      </c>
+      <c r="F31" s="9">
+        <f>D31+E31</f>
+        <v/>
+      </c>
+      <c r="G31" s="29">
+        <f>IF(F31=0,"",E31/F31)</f>
+        <v/>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>メーカー事務系</t>
+        </is>
+      </c>
+      <c r="I31" s="27" t="inlineStr">
+        <is>
+          <t>事務系コース内定者の比率（%）。技術系は理系100%。唯一見つかったメーカー事務系の直接データ</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>三菱商事</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="n">
+        <v>108</v>
+      </c>
+      <c r="E32" s="19" t="n">
+        <v>31</v>
+      </c>
+      <c r="F32" s="18">
+        <f>D32+E32</f>
+        <v/>
+      </c>
+      <c r="G32" s="30">
+        <f>IF(F32=0,"",E32/F32)</f>
+        <v/>
+      </c>
+      <c r="H32" s="18" t="inlineStr">
+        <is>
+          <t>商社（全員ビジネス職）</t>
+        </is>
+      </c>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>技術系の枠がないため、理系も全員ビジネス職</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>伊藤忠商事</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="n">
+        <v>96</v>
+      </c>
+      <c r="E33" s="19" t="n">
+        <v>38</v>
+      </c>
+      <c r="F33" s="18">
+        <f>D33+E33</f>
+        <v/>
+      </c>
+      <c r="G33" s="30">
+        <f>IF(F33=0,"",E33/F33)</f>
+        <v/>
+      </c>
+      <c r="H33" s="18" t="inlineStr">
+        <is>
+          <t>商社（全員ビジネス職）</t>
+        </is>
+      </c>
+      <c r="I33" s="16" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>三菱UFJ銀行</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>最新</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="n">
+        <v>80</v>
+      </c>
+      <c r="E34" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="F34" s="18">
+        <f>D34+E34</f>
+        <v/>
+      </c>
+      <c r="G34" s="30">
+        <f>IF(F34=0,"",E34/F34)</f>
+        <v/>
+      </c>
+      <c r="H34" s="18" t="inlineStr">
+        <is>
+          <t>銀行</t>
+        </is>
+      </c>
+      <c r="I34" s="16" t="inlineStr">
+        <is>
+          <t>「内定の2割が理系」（ニッキン報道）。デジタル等の専門コース込み</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>・富士フイルムBIの行は人数ではなく%（合計100）。商社・銀行は技術系の枠がない分、理系がビジネス職に流れるので、メーカー事務系より理系比率が高めに出ます。</t>
         </is>
       </c>
     </row>
@@ -8384,77 +8592,77 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="34" t="inlineStr">
+      <c r="B1" s="35" t="inlineStr">
         <is>
           <t>業界（プルダウンの選択肢。追加・変更OK）</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="35" t="inlineStr">
+      <c r="B2" s="36" t="inlineStr">
         <is>
           <t>コンサル</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="35" t="inlineStr">
+      <c r="B3" s="36" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="35" t="inlineStr">
+      <c r="B4" s="36" t="inlineStr">
         <is>
           <t>人材・広告</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="35" t="inlineStr">
+      <c r="B5" s="36" t="inlineStr">
         <is>
           <t>鉄鋼・素材</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="35" t="inlineStr">
+      <c r="B6" s="36" t="inlineStr">
         <is>
           <t>化学</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="35" t="inlineStr">
+      <c r="B7" s="36" t="inlineStr">
         <is>
           <t>プラント・エンジ</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="35" t="inlineStr">
+      <c r="B8" s="36" t="inlineStr">
         <is>
           <t>技術営業</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="35" t="inlineStr">
+      <c r="B9" s="36" t="inlineStr">
         <is>
           <t>半導体・電機メーカー</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="35" t="inlineStr">
+      <c r="B10" s="36" t="inlineStr">
         <is>
           <t>商社</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="35" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>その他</t>
         </is>

</xml_diff>